<commit_message>
feat(materials): streamline spreadsheet library workflow
</commit_message>
<xml_diff>
--- a/src/inductor_designer/resources/material_templates/material-import-template.xlsx
+++ b/src/inductor_designer/resources/material_templates/material-import-template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rbd83f437409c48b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material" sheetId="2" r:id="Rf6cae557d5174e5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B-H Curves" sheetId="3" r:id="Rc6624cdce7d44c01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loss Curves" sheetId="4" r:id="Rfa426eaf38fe46a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Ra0638230dc2d45a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material" sheetId="2" r:id="Racf1812310a1466d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B-H Curves" sheetId="3" r:id="R645eb600457f4a57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loss Curves" sheetId="4" r:id="R1b5fcf87b6f04505"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -558,28 +558,28 @@
         <x:v>Replace or delete every synthetic example row, enter source metadata, then upload the completed workbook for validation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
+    <x:row r="5" ht="30" hidden="0" customHeight="1">
       <x:c r="A5" s="16" t="str">
         <x:v>Required metadata</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
-        <x:v>Manufacturer, material name, grade, capture timestamp, and source description are required. Source URL and page may be blank.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+        <x:v>Manufacturer, material name, grade, and source description are required. Enter capture date/time as text or an Excel date; date cells are normalized to ISO on import. Source URL and page may be blank.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="30" hidden="0" customHeight="1">
       <x:c r="A6" s="16" t="str">
         <x:v>B-H series</x:v>
       </x:c>
       <x:c r="B6" s="17" t="str">
-        <x:v>Rows sharing series_id must repeat identical temperature, DC bias, and units. H units: A/m, kA/m, Oe. B units: T, mT, G, kG.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+        <x:v>Rows sharing series_id must repeat identical temperature, DC bias, and units. DC bias is optional; leave blank when source does not report it. H units: A/m, kA/m, Oe. B units: T, mT, G, kG.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="30" hidden="0" customHeight="1">
       <x:c r="A7" s="16" t="str">
         <x:v>Loss series</x:v>
       </x:c>
       <x:c r="B7" s="17" t="str">
-        <x:v>Frequency must be positive. Rows sharing series_id must repeat identical frequency, temperature, DC bias, and units.</x:v>
+        <x:v>Frequency must be positive. Rows sharing series_id must repeat identical frequency, temperature, DC bias, and units. DC bias is optional; 0 means explicitly measured without DC bias.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -689,7 +689,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raea4d5687e6c4dd6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f98bed796a54617"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -718,16 +718,16 @@
         <x:v>dc_bias_a_per_m</x:v>
       </x:c>
       <x:c r="D1" s="7" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="E1" s="7" t="str">
         <x:v>h_unit</x:v>
       </x:c>
-      <x:c r="E1" s="7" t="str">
+      <x:c r="F1" s="7" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="G1" s="7" t="str">
         <x:v>b_unit</x:v>
-      </x:c>
-      <x:c r="F1" s="7" t="str">
-        <x:v>h</x:v>
-      </x:c>
-      <x:c r="G1" s="7" t="str">
-        <x:v>b</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -738,17 +738,17 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="C2" s="37"/>
-      <x:c r="D2" s="29" t="str">
+      <x:c r="D2" s="29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E2" s="29" t="str">
         <x:v>Oe</x:v>
-      </x:c>
-      <x:c r="E2" s="29" t="str">
-        <x:v>kG</x:v>
       </x:c>
       <x:c r="F2" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G2" s="41" t="n">
-        <x:v>0</x:v>
+      <x:c r="G2" s="41" t="str">
+        <x:v>kG</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -759,17 +759,17 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="C3" s="38"/>
-      <x:c r="D3" s="32" t="str">
+      <x:c r="D3" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E3" s="32" t="str">
         <x:v>Oe</x:v>
-      </x:c>
-      <x:c r="E3" s="32" t="str">
-        <x:v>kG</x:v>
       </x:c>
       <x:c r="F3" s="42" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G3" s="43" t="n">
-        <x:v>1</x:v>
+      <x:c r="G3" s="43" t="str">
+        <x:v>kG</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -780,31 +780,31 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="C4" s="39"/>
-      <x:c r="D4" s="35" t="str">
+      <x:c r="D4" s="35" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E4" s="35" t="str">
         <x:v>Oe</x:v>
       </x:c>
-      <x:c r="E4" s="35" t="str">
+      <x:c r="F4" s="44" t="n">
+        <x:v>1.6</x:v>
+      </x:c>
+      <x:c r="G4" s="45" t="str">
         <x:v>kG</x:v>
-      </x:c>
-      <x:c r="F4" s="44" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G4" s="45" t="n">
-        <x:v>1.6</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="D2:D200">
+    <x:dataValidation type="list" sqref="E2:E200">
       <x:formula1>"A/m,kA/m,Oe"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="E2:E200">
+    <x:dataValidation type="list" sqref="G2:G200">
       <x:formula1>"T,mT,G,kG"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac2fc34352bf4d15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R733dc109a65e42ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -837,16 +837,16 @@
         <x:v>dc_bias_a_per_m</x:v>
       </x:c>
       <x:c r="E1" s="7" t="str">
+        <x:v>b</x:v>
+      </x:c>
+      <x:c r="F1" s="7" t="str">
         <x:v>b_unit</x:v>
       </x:c>
-      <x:c r="F1" s="7" t="str">
+      <x:c r="G1" s="7" t="str">
+        <x:v>loss</x:v>
+      </x:c>
+      <x:c r="H1" s="7" t="str">
         <x:v>loss_unit</x:v>
-      </x:c>
-      <x:c r="G1" s="7" t="str">
-        <x:v>b</x:v>
-      </x:c>
-      <x:c r="H1" s="7" t="str">
-        <x:v>loss</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -862,17 +862,17 @@
       <x:c r="D2" s="37" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E2" s="29" t="str">
+      <x:c r="E2" s="29" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F2" s="29" t="str">
         <x:v>kG</x:v>
       </x:c>
-      <x:c r="F2" s="29" t="str">
+      <x:c r="G2" s="40" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="H2" s="41" t="str">
         <x:v>mW/cm3</x:v>
-      </x:c>
-      <x:c r="G2" s="40" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="H2" s="41" t="n">
-        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -888,17 +888,17 @@
       <x:c r="D3" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E3" s="32" t="str">
+      <x:c r="E3" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F3" s="32" t="str">
         <x:v>kG</x:v>
       </x:c>
-      <x:c r="F3" s="32" t="str">
+      <x:c r="G3" s="42" t="n">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="H3" s="43" t="str">
         <x:v>mW/cm3</x:v>
-      </x:c>
-      <x:c r="G3" s="42" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H3" s="43" t="n">
-        <x:v>240</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -914,17 +914,17 @@
       <x:c r="D4" s="38" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E4" s="32" t="str">
+      <x:c r="E4" s="32" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F4" s="32" t="str">
         <x:v>kG</x:v>
       </x:c>
-      <x:c r="F4" s="32" t="str">
+      <x:c r="G4" s="42" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="H4" s="43" t="str">
         <x:v>mW/cm3</x:v>
-      </x:c>
-      <x:c r="G4" s="42" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="H4" s="43" t="n">
-        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -940,31 +940,31 @@
       <x:c r="D5" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E5" s="35" t="str">
+      <x:c r="E5" s="35" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F5" s="35" t="str">
         <x:v>kG</x:v>
       </x:c>
-      <x:c r="F5" s="35" t="str">
+      <x:c r="G5" s="44" t="n">
+        <x:v>430</x:v>
+      </x:c>
+      <x:c r="H5" s="45" t="str">
         <x:v>mW/cm3</x:v>
-      </x:c>
-      <x:c r="G5" s="44" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H5" s="45" t="n">
-        <x:v>430</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="E2:E200">
+    <x:dataValidation type="list" sqref="F2:F200">
       <x:formula1>"T,mT,G,kG"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="F2:F200">
+    <x:dataValidation type="list" sqref="H2:H200">
       <x:formula1>"W/m3,kW/m3,mW/cm3"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6df310ec373410f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dd6d7ba80734e20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>